<commit_message>
Update mods and config
</commit_message>
<xml_diff>
--- a/config/reskillable/расчёты.xlsx
+++ b/config/reskillable/расчёты.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Minecraft\profiles\TechnoVanilla 1.1.2\config\reskillable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Minecraft\profiles\TechnoVanilla 1.1.4\config\reskillable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11338AD-FE2D-407D-93A2-33F96290DE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FF9060-A401-4DCF-BA10-4326C47EC0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -419,17 +419,17 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>6</v>
+        <v>8.4</v>
       </c>
       <c r="B3" s="1">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" s="1">
         <f>(A3*B3)-4+(C3*2)</f>
-        <v>9.6000000000000014</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>

</xml_diff>

<commit_message>
Update config and toml for the Reskil Lable mod
</commit_message>
<xml_diff>
--- a/config/reskillable/расчёты.xlsx
+++ b/config/reskillable/расчёты.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Minecraft\profiles\TechnoVanilla 1.1.4\config\reskillable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FF9060-A401-4DCF-BA10-4326C47EC0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EAEB2A0-400D-4883-BB57-D53BAA369CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,13 +66,13 @@
     <t>от 200 до 499</t>
   </si>
   <si>
-    <t>от 500 до 999</t>
-  </si>
-  <si>
-    <t>1000+</t>
-  </si>
-  <si>
     <t>до 199</t>
+  </si>
+  <si>
+    <t>от 500 до 999+</t>
+  </si>
+  <si>
+    <t>неломаемое</t>
   </si>
 </sst>
 </file>
@@ -419,17 +419,17 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>8.4</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1">
         <f>(A3*B3)-4+(C3*2)</f>
-        <v>4.4000000000000004</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -458,17 +458,17 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1">
         <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D7" s="1">
         <f>(A7+B7)*1</f>
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -477,25 +477,25 @@
       </c>
       <c r="D8" s="1">
         <f>(A7+B7)*2</f>
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1">
         <f>(A7+B7)*3</f>
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="1">
         <f>(A7+B7)*4</f>
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V1.2.0.2 Update mod + bag fix + Update quest
</commit_message>
<xml_diff>
--- a/config/reskillable/расчёты.xlsx
+++ b/config/reskillable/расчёты.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Minecraft\profiles\TechnoVanilla 1.1.4\config\reskillable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AF6ACE-56EE-43BF-BB13-9F53E4AD25F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76121DFD-D9C8-45DC-88D0-0F06B6E7CCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -419,17 +419,17 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
       </c>
       <c r="D3" s="1">
         <f>(A3*B3)-4+(C3*2)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>

</xml_diff>